<commit_message>
Make Clover Product Codes authoritative to Big Fireworks UPC list
Per decision to trust the Big spreadsheet, every confidently name-matched
item now carries Big's UPC. Net vs original export: 117 blanks filled, 37
existing codes corrected to Big (including fixing wrong CF-derived codes
from earlier steps), 4 codes cleared where Big assigns that barcode to a
different product. No other columns changed. Added a change-log workbook
listing all 158 Product Code changes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FR35jspmg12CbjyrmrWzCK
</commit_message>
<xml_diff>
--- a/inventoryexportv2_1_updated.xlsx
+++ b/inventoryexportv2_1_updated.xlsx
@@ -249,7 +249,7 @@
     <xf numFmtId="0" fontId="40" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="40" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -372,6 +372,9 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="42" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3010,7 +3013,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>813559002452</t>
+          <t>847294034553</t>
         </is>
       </c>
       <c r="J30" s="2" t="n"/>
@@ -3120,7 +3123,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>000000110426</t>
+          <t>8472940071201</t>
         </is>
       </c>
       <c r="J32" s="2" t="n"/>
@@ -3169,7 +3172,7 @@
       <c r="H33" s="1" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>847294007120</t>
+          <t>8472940071201</t>
         </is>
       </c>
       <c r="J33" s="2" t="n"/>
@@ -3572,7 +3575,11 @@
         </is>
       </c>
       <c r="H41" s="1" t="inlineStr"/>
-      <c r="I41" s="2" t="n"/>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>676821102836</t>
+        </is>
+      </c>
       <c r="J41" s="2" t="n"/>
       <c r="K41" s="2" t="inlineStr"/>
       <c r="L41" s="2" t="inlineStr">
@@ -4687,7 +4694,11 @@
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr"/>
-      <c r="I62" s="2" t="n"/>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>847294014050</t>
+        </is>
+      </c>
       <c r="J62" s="2" t="n"/>
       <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr">
@@ -5890,7 +5901,11 @@
         </is>
       </c>
       <c r="H85" s="1" t="inlineStr"/>
-      <c r="I85" s="2" t="n"/>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>847294004709</t>
+        </is>
+      </c>
       <c r="J85" s="2" t="n"/>
       <c r="K85" s="2" t="inlineStr"/>
       <c r="L85" s="2" t="inlineStr">
@@ -6007,11 +6022,7 @@
       <c r="H87" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="I87" s="2" t="inlineStr">
-        <is>
-          <t>847294039251</t>
-        </is>
-      </c>
+      <c r="I87" s="2" t="n"/>
       <c r="J87" s="2" t="n"/>
       <c r="K87" s="2" t="inlineStr"/>
       <c r="L87" s="2" t="inlineStr">
@@ -6363,7 +6374,11 @@
         </is>
       </c>
       <c r="H94" s="1" t="inlineStr"/>
-      <c r="I94" s="2" t="n"/>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>847294039251</t>
+        </is>
+      </c>
       <c r="J94" s="2" t="n"/>
       <c r="K94" s="2" t="inlineStr"/>
       <c r="L94" s="2" t="inlineStr">
@@ -6726,7 +6741,7 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>47294095325</t>
+          <t>847294095325</t>
         </is>
       </c>
       <c r="J101" s="2" t="n"/>
@@ -7444,7 +7459,7 @@
       <c r="H114" s="1" t="inlineStr"/>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>6950165406657</t>
+          <t>847294016825</t>
         </is>
       </c>
       <c r="J114" s="2" t="n"/>
@@ -8156,7 +8171,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>729205027895</t>
+          <t>847294045207</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -8722,7 +8737,7 @@
       <c r="H139" s="1" t="inlineStr"/>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>847294016825</t>
+          <t>847294094571</t>
         </is>
       </c>
       <c r="J139" s="2" t="n"/>
@@ -9047,7 +9062,7 @@
       <c r="H145" s="1" t="inlineStr"/>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>601527870376</t>
+          <t>601527824386</t>
         </is>
       </c>
       <c r="J145" s="2" t="n"/>
@@ -11720,7 +11735,7 @@
       <c r="H193" s="1" t="inlineStr"/>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>676821258557</t>
+          <t>847294008622</t>
         </is>
       </c>
       <c r="J193" s="2" t="n"/>
@@ -12541,7 +12556,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>47294090498</t>
+          <t>847294004648</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -13681,7 +13696,7 @@
       <c r="H229" s="1" t="inlineStr"/>
       <c r="I229" s="2" t="inlineStr">
         <is>
-          <t>847294089058</t>
+          <t>847294020167</t>
         </is>
       </c>
       <c r="J229" s="2" t="n"/>
@@ -13852,7 +13867,7 @@
       <c r="H232" s="1" t="inlineStr"/>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>847294041124</t>
+          <t>847294029184</t>
         </is>
       </c>
       <c r="J232" s="2" t="n"/>
@@ -14237,7 +14252,11 @@
         </is>
       </c>
       <c r="H239" s="1" t="inlineStr"/>
-      <c r="I239" s="2" t="n"/>
+      <c r="I239" s="2" t="inlineStr">
+        <is>
+          <t>847294094991</t>
+        </is>
+      </c>
       <c r="J239" s="2" t="n"/>
       <c r="K239" s="2" t="inlineStr"/>
       <c r="L239" s="2" t="inlineStr">
@@ -15003,7 +15022,11 @@
         </is>
       </c>
       <c r="H253" s="1" t="inlineStr"/>
-      <c r="I253" s="2" t="n"/>
+      <c r="I253" s="2" t="inlineStr">
+        <is>
+          <t>676821258557</t>
+        </is>
+      </c>
       <c r="J253" s="2" t="n"/>
       <c r="K253" s="2" t="inlineStr"/>
       <c r="L253" s="2" t="inlineStr">
@@ -15726,7 +15749,7 @@
       <c r="H266" s="1" t="inlineStr"/>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>847294004709</t>
+          <t>676821085986</t>
         </is>
       </c>
       <c r="J266" s="2" t="n"/>
@@ -17667,11 +17690,7 @@
         </is>
       </c>
       <c r="H303" s="1" t="inlineStr"/>
-      <c r="I303" s="2" t="inlineStr">
-        <is>
-          <t>676821310378</t>
-        </is>
-      </c>
+      <c r="I303" s="2" t="n"/>
       <c r="J303" s="2" t="n"/>
       <c r="K303" s="2" t="inlineStr"/>
       <c r="L303" s="2" t="inlineStr">
@@ -20246,7 +20265,7 @@
       <c r="H352" s="1" t="inlineStr"/>
       <c r="I352" s="2" t="inlineStr">
         <is>
-          <t>676821085986</t>
+          <t>847294009049</t>
         </is>
       </c>
       <c r="J352" s="2" t="n"/>
@@ -20356,7 +20375,7 @@
       <c r="H354" s="1" t="inlineStr"/>
       <c r="I354" s="2" t="inlineStr">
         <is>
-          <t>676821077042</t>
+          <t>847294085586</t>
         </is>
       </c>
       <c r="J354" s="2" t="n"/>
@@ -20475,7 +20494,7 @@
       <c r="H356" s="1" t="inlineStr"/>
       <c r="I356" s="2" t="inlineStr">
         <is>
-          <t>847294042039</t>
+          <t>847294085593</t>
         </is>
       </c>
       <c r="J356" s="2" t="n"/>
@@ -20594,7 +20613,7 @@
       <c r="H358" s="1" t="inlineStr"/>
       <c r="I358" s="2" t="inlineStr">
         <is>
-          <t>676821433930</t>
+          <t>847294085647</t>
         </is>
       </c>
       <c r="J358" s="2" t="n"/>
@@ -23022,7 +23041,7 @@
       </c>
       <c r="I402" s="2" t="inlineStr">
         <is>
-          <t>950165402499</t>
+          <t>6950165407499</t>
         </is>
       </c>
       <c r="J402" s="2" t="n"/>
@@ -23138,7 +23157,7 @@
       </c>
       <c r="I404" s="2" t="inlineStr">
         <is>
-          <t>950165402482</t>
+          <t>6950165407499</t>
         </is>
       </c>
       <c r="J404" s="2" t="n"/>
@@ -23567,7 +23586,7 @@
       <c r="H412" s="1" t="inlineStr"/>
       <c r="I412" s="2" t="inlineStr">
         <is>
-          <t>6950165415840</t>
+          <t>847294031453</t>
         </is>
       </c>
       <c r="J412" s="2" t="n"/>
@@ -23678,7 +23697,7 @@
       </c>
       <c r="I414" s="2" t="inlineStr">
         <is>
-          <t>875330061706</t>
+          <t>676821143167</t>
         </is>
       </c>
       <c r="J414" s="2" t="inlineStr">
@@ -24412,7 +24431,7 @@
       <c r="H428" s="1" t="inlineStr"/>
       <c r="I428" s="2" t="inlineStr">
         <is>
-          <t>676821266873</t>
+          <t>847294042039</t>
         </is>
       </c>
       <c r="J428" s="2" t="n"/>
@@ -24714,7 +24733,7 @@
       </c>
       <c r="I434" s="2" t="inlineStr">
         <is>
-          <t>847294031019</t>
+          <t>847294031002</t>
         </is>
       </c>
       <c r="J434" s="2" t="n"/>
@@ -24768,7 +24787,7 @@
       <c r="H435" s="1" t="inlineStr"/>
       <c r="I435" s="2" t="inlineStr">
         <is>
-          <t>847294031019</t>
+          <t>847294031002</t>
         </is>
       </c>
       <c r="J435" s="2" t="n"/>
@@ -26287,7 +26306,7 @@
       </c>
       <c r="I463" s="2" t="inlineStr">
         <is>
-          <t>8145270502815</t>
+          <t>847294036984</t>
         </is>
       </c>
       <c r="J463" s="2" t="inlineStr">
@@ -29481,7 +29500,7 @@
       </c>
       <c r="I522" s="2" t="inlineStr">
         <is>
-          <t>875330063908</t>
+          <t>676821135438</t>
         </is>
       </c>
       <c r="J522" s="2" t="inlineStr">
@@ -30014,7 +30033,11 @@
         </is>
       </c>
       <c r="H532" s="1" t="inlineStr"/>
-      <c r="I532" s="2" t="n"/>
+      <c r="I532" s="2" t="inlineStr">
+        <is>
+          <t>676821439659</t>
+        </is>
+      </c>
       <c r="J532" s="2" t="n"/>
       <c r="K532" s="2" t="inlineStr"/>
       <c r="L532" s="2" t="inlineStr">
@@ -30129,7 +30152,11 @@
         </is>
       </c>
       <c r="H534" s="1" t="inlineStr"/>
-      <c r="I534" s="2" t="n"/>
+      <c r="I534" s="2" t="inlineStr">
+        <is>
+          <t>676821433930</t>
+        </is>
+      </c>
       <c r="J534" s="2" t="n"/>
       <c r="K534" s="2" t="inlineStr"/>
       <c r="L534" s="2" t="inlineStr">
@@ -32076,7 +32103,11 @@
         </is>
       </c>
       <c r="H571" s="1" t="inlineStr"/>
-      <c r="I571" s="2" t="n"/>
+      <c r="I571" s="2" t="inlineStr">
+        <is>
+          <t>847294009254</t>
+        </is>
+      </c>
       <c r="J571" s="2" t="n"/>
       <c r="K571" s="2" t="inlineStr"/>
       <c r="L571" s="2" t="inlineStr">
@@ -33188,7 +33219,7 @@
       </c>
       <c r="I592" s="2" t="inlineStr">
         <is>
-          <t>47294092485</t>
+          <t>847294092485</t>
         </is>
       </c>
       <c r="J592" s="2" t="n"/>
@@ -33394,7 +33425,7 @@
       <c r="H596" s="1" t="inlineStr"/>
       <c r="I596" s="2" t="inlineStr">
         <is>
-          <t>193836410928</t>
+          <t>676821059819</t>
         </is>
       </c>
       <c r="J596" s="2" t="n"/>
@@ -33672,7 +33703,7 @@
       </c>
       <c r="I601" s="2" t="inlineStr">
         <is>
-          <t>676821122988</t>
+          <t>676821310378</t>
         </is>
       </c>
       <c r="J601" s="2" t="n"/>
@@ -36521,7 +36552,7 @@
       </c>
       <c r="I657" s="2" t="inlineStr">
         <is>
-          <t>193836404620</t>
+          <t>847294041926</t>
         </is>
       </c>
       <c r="J657" s="2" t="n"/>
@@ -36577,7 +36608,7 @@
       <c r="H658" s="1" t="inlineStr"/>
       <c r="I658" s="2" t="inlineStr">
         <is>
-          <t>47294041926</t>
+          <t>847294041926</t>
         </is>
       </c>
       <c r="J658" s="2" t="n"/>
@@ -36628,7 +36659,7 @@
       <c r="H659" s="1" t="inlineStr"/>
       <c r="I659" s="2" t="inlineStr">
         <is>
-          <t>676821102836</t>
+          <t>847294041926</t>
         </is>
       </c>
       <c r="J659" s="2" t="n"/>
@@ -41003,11 +41034,7 @@
         </is>
       </c>
       <c r="H743" s="1" t="inlineStr"/>
-      <c r="I743" s="2" t="inlineStr">
-        <is>
-          <t>676821439659</t>
-        </is>
-      </c>
+      <c r="I743" s="2" t="n"/>
       <c r="J743" s="2" t="n"/>
       <c r="K743" s="2" t="inlineStr"/>
       <c r="L743" s="2" t="inlineStr">
@@ -43040,11 +43067,7 @@
         </is>
       </c>
       <c r="H782" s="1" t="inlineStr"/>
-      <c r="I782" s="2" t="inlineStr">
-        <is>
-          <t>847294001463</t>
-        </is>
-      </c>
+      <c r="I782" s="2" t="n"/>
       <c r="J782" s="2" t="n"/>
       <c r="K782" s="2" t="inlineStr"/>
       <c r="L782" s="2" t="inlineStr">
@@ -43899,7 +43922,7 @@
       </c>
       <c r="I801" s="2" t="inlineStr">
         <is>
-          <t>6950165409283</t>
+          <t>847294025391</t>
         </is>
       </c>
       <c r="J801" s="2" t="inlineStr">
@@ -45142,7 +45165,7 @@
       </c>
       <c r="I826" s="2" t="inlineStr">
         <is>
-          <t>847294016849</t>
+          <t>847294096469</t>
         </is>
       </c>
       <c r="J826" s="2" t="inlineStr">
@@ -45307,7 +45330,11 @@
         </is>
       </c>
       <c r="H829" s="1" t="inlineStr"/>
-      <c r="I829" s="2" t="n"/>
+      <c r="I829" s="2" t="inlineStr">
+        <is>
+          <t>6950165415840</t>
+        </is>
+      </c>
       <c r="J829" s="2" t="n"/>
       <c r="K829" s="2" t="inlineStr"/>
       <c r="L829" s="2" t="inlineStr">
@@ -45677,7 +45704,7 @@
       </c>
       <c r="I836" s="2" t="inlineStr">
         <is>
-          <t>652009003409</t>
+          <t>847294019116</t>
         </is>
       </c>
       <c r="J836" s="2" t="inlineStr">
@@ -46275,7 +46302,7 @@
       </c>
       <c r="I847" s="2" t="inlineStr">
         <is>
-          <t>145270102121</t>
+          <t>676821186195</t>
         </is>
       </c>
       <c r="J847" s="2" t="n"/>
@@ -49563,7 +49590,7 @@
       </c>
       <c r="I915" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>676821266873</t>
         </is>
       </c>
       <c r="J915" s="2" t="n"/>
@@ -49662,7 +49689,7 @@
       <c r="H917" s="1" t="inlineStr"/>
       <c r="I917" s="2" t="inlineStr">
         <is>
-          <t>847294014050</t>
+          <t>676821266873</t>
         </is>
       </c>
       <c r="J917" s="2" t="n"/>
@@ -50393,7 +50420,7 @@
       <c r="H930" s="1" t="inlineStr"/>
       <c r="I930" s="2" t="inlineStr">
         <is>
-          <t>753459922682</t>
+          <t>676821106629</t>
         </is>
       </c>
       <c r="J930" s="2" t="n"/>
@@ -53101,7 +53128,7 @@
       <c r="H985" s="1" t="inlineStr"/>
       <c r="I985" s="2" t="inlineStr">
         <is>
-          <t>813559007501</t>
+          <t>847294030920</t>
         </is>
       </c>
       <c r="J985" s="2" t="n"/>
@@ -54136,7 +54163,11 @@
         </is>
       </c>
       <c r="H1005" s="1" t="inlineStr"/>
-      <c r="I1005" s="2" t="n"/>
+      <c r="I1005" s="2" t="inlineStr">
+        <is>
+          <t>847294085982</t>
+        </is>
+      </c>
       <c r="J1005" s="2" t="n"/>
       <c r="K1005" s="2" t="inlineStr"/>
       <c r="L1005" s="2" t="inlineStr">
@@ -55265,7 +55296,7 @@
       <c r="H1027" s="1" t="inlineStr"/>
       <c r="I1027" s="2" t="inlineStr">
         <is>
-          <t>875330020208</t>
+          <t>847294092423</t>
         </is>
       </c>
       <c r="J1027" s="2" t="n"/>
@@ -55316,7 +55347,7 @@
       </c>
       <c r="I1028" s="2" t="inlineStr">
         <is>
-          <t>75330020208</t>
+          <t>847294092423</t>
         </is>
       </c>
       <c r="J1028" s="2" t="n"/>
@@ -56450,7 +56481,7 @@
       </c>
       <c r="I1049" s="2" t="inlineStr">
         <is>
-          <t>695016540307</t>
+          <t>6950165403014</t>
         </is>
       </c>
       <c r="J1049" s="2" t="inlineStr">
@@ -57768,8 +57799,10 @@
       <c r="H1075" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="I1075" s="44" t="n">
-        <v>847294098395</v>
+      <c r="I1075" s="48" t="inlineStr">
+        <is>
+          <t>676821466891</t>
+        </is>
       </c>
       <c r="J1075" s="44" t="n">
         <v>847294098395</v>
@@ -57919,7 +57952,7 @@
       <c r="H1078" s="1" t="inlineStr"/>
       <c r="I1078" s="2" t="inlineStr">
         <is>
-          <t>847294012124</t>
+          <t>676821478092</t>
         </is>
       </c>
       <c r="J1078" s="2" t="n"/>
@@ -58713,11 +58746,7 @@
       <c r="H1096" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="I1096" s="2" t="inlineStr">
-        <is>
-          <t>847294042022</t>
-        </is>
-      </c>
+      <c r="I1096" s="2" t="n"/>
       <c r="J1096" s="2" t="inlineStr">
         <is>
           <t>847294042022</t>
@@ -62334,7 +62363,7 @@
       <c r="H1165" s="1" t="inlineStr"/>
       <c r="I1165" s="2" t="inlineStr">
         <is>
-          <t>47294013145</t>
+          <t>847294013145</t>
         </is>
       </c>
       <c r="J1165" s="2" t="n"/>
@@ -63166,7 +63195,7 @@
       <c r="H1181" s="1" t="inlineStr"/>
       <c r="I1181" s="2" t="inlineStr">
         <is>
-          <t>6950165409382</t>
+          <t>847294008042</t>
         </is>
       </c>
       <c r="J1181" s="2" t="n"/>
@@ -63630,7 +63659,7 @@
       </c>
       <c r="I1190" s="2" t="inlineStr">
         <is>
-          <t>6944112605170</t>
+          <t>805253516328</t>
         </is>
       </c>
       <c r="J1190" s="2" t="inlineStr">
@@ -63683,7 +63712,7 @@
       <c r="H1191" s="1" t="inlineStr"/>
       <c r="I1191" s="2" t="inlineStr">
         <is>
-          <t>847294029184</t>
+          <t>847294004129</t>
         </is>
       </c>
       <c r="J1191" s="2" t="n"/>
@@ -64467,7 +64496,7 @@
       <c r="H1206" s="1" t="inlineStr"/>
       <c r="I1206" s="2" t="inlineStr">
         <is>
-          <t>47294040332</t>
+          <t>6950165408477</t>
         </is>
       </c>
       <c r="J1206" s="2" t="n"/>
@@ -65463,7 +65492,7 @@
       </c>
       <c r="I1225" s="2" t="inlineStr">
         <is>
-          <t>950165407098</t>
+          <t>6944112600366</t>
         </is>
       </c>
       <c r="J1225" s="2" t="n"/>
@@ -66663,7 +66692,7 @@
       <c r="H1248" s="1" t="inlineStr"/>
       <c r="I1248" s="2" t="inlineStr">
         <is>
-          <t>847294039022</t>
+          <t>676821374431</t>
         </is>
       </c>
       <c r="J1248" s="2" t="n"/>
@@ -67783,7 +67812,7 @@
       <c r="H1271" s="1" t="inlineStr"/>
       <c r="I1271" s="2" t="inlineStr">
         <is>
-          <t>847294006178</t>
+          <t>847294008417</t>
         </is>
       </c>
       <c r="J1271" s="2" t="n"/>
@@ -68102,7 +68131,7 @@
       <c r="H1277" s="1" t="inlineStr"/>
       <c r="I1277" s="2" t="inlineStr">
         <is>
-          <t>847294094991</t>
+          <t>847294096315</t>
         </is>
       </c>
       <c r="J1277" s="2" t="n"/>
@@ -71559,7 +71588,7 @@
       </c>
       <c r="I1342" s="2" t="inlineStr">
         <is>
-          <t>847294017075</t>
+          <t>847294092515</t>
         </is>
       </c>
       <c r="J1342" s="2" t="inlineStr">
@@ -71667,8 +71696,10 @@
           <t>Home Run</t>
         </is>
       </c>
-      <c r="I1346" s="45" t="n">
-        <v>193836410928</v>
+      <c r="I1346" s="2" t="inlineStr">
+        <is>
+          <t>676821059819</t>
+        </is>
       </c>
     </row>
     <row r="1347">
@@ -71720,9 +71751,7 @@
           <t>Captain Marvel</t>
         </is>
       </c>
-      <c r="I1352" s="45" t="n">
-        <v>847294030272</v>
-      </c>
+      <c r="I1352" s="45" t="n"/>
     </row>
     <row r="1353">
       <c r="B1353" t="inlineStr">
@@ -71840,8 +71869,10 @@
           <t>blast zone</t>
         </is>
       </c>
-      <c r="I1364" s="45" t="n">
-        <v>753459937747</v>
+      <c r="I1364" s="2" t="inlineStr">
+        <is>
+          <t>676821076113</t>
+        </is>
       </c>
     </row>
     <row r="1365">

</xml_diff>

<commit_message>
Fill THE PERFECT MATCH with Raccoon item UPC from official site
Sourced 757205301226 from raccoonfireworksusa.com product page (Raccoon
757205 item-UPC prefix). Web-sourced; recommend visual verification.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FR35jspmg12CbjyrmrWzCK
</commit_message>
<xml_diff>
--- a/inventoryexportv2_1_updated.xlsx
+++ b/inventoryexportv2_1_updated.xlsx
@@ -65132,7 +65132,11 @@
         </is>
       </c>
       <c r="H1218" s="1" t="inlineStr"/>
-      <c r="I1218" s="2" t="n"/>
+      <c r="I1218" s="2" t="inlineStr">
+        <is>
+          <t>757205301226</t>
+        </is>
+      </c>
       <c r="J1218" s="2" t="n"/>
       <c r="K1218" s="2" t="inlineStr"/>
       <c r="L1218" s="2" t="inlineStr">

</xml_diff>